<commit_message>
changes to text by ChrisW
</commit_message>
<xml_diff>
--- a/paper/Tables/fs_treatment_effects.xlsx
+++ b/paper/Tables/fs_treatment_effects.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24931"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25330"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\isaac\Dropbox\ReplicationFinal\Tables\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\isaac\Dropbox\Apps\ShareLaTeX\Information Settlement_2020\paper\Tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BC24273-5BEA-4097-804F-23746D210366}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EAFDEAB-46AD-4855-BCC8-289C7DF21F99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{DFE3BC43-0C70-43BF-BB5D-76E96627C8A4}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
   <si>
     <t>R-squared</t>
   </si>
@@ -53,9 +53,6 @@
   </si>
   <si>
     <t xml:space="preserve">Calculator </t>
-  </si>
-  <si>
-    <t>Settlement</t>
   </si>
   <si>
     <t>Emp present</t>
@@ -74,6 +71,18 @@
   </si>
   <si>
     <t>Conditional on EP=0</t>
+  </si>
+  <si>
+    <t>(1)</t>
+  </si>
+  <si>
+    <t>(2)</t>
+  </si>
+  <si>
+    <t>(3)</t>
+  </si>
+  <si>
+    <t>(4)</t>
   </si>
 </sst>
 </file>
@@ -138,7 +147,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -163,6 +172,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -194,42 +206,12 @@
           <cell r="A2" t="str">
             <v/>
           </cell>
-          <cell r="B2" t="str">
-            <v>(1)</v>
-          </cell>
-          <cell r="C2" t="str">
-            <v>(2)</v>
-          </cell>
-          <cell r="D2" t="str">
-            <v>(3)</v>
-          </cell>
-          <cell r="E2" t="str">
-            <v>(4)</v>
-          </cell>
-          <cell r="F2" t="str">
-            <v>(5)</v>
-          </cell>
-          <cell r="G2" t="str">
-            <v>(6)</v>
-          </cell>
-          <cell r="H2" t="str">
-            <v>(7)</v>
-          </cell>
         </row>
         <row r="9">
-          <cell r="B9" t="str">
-            <v>0.121</v>
-          </cell>
           <cell r="C9" t="str">
             <v/>
           </cell>
           <cell r="D9" t="str">
-            <v/>
-          </cell>
-          <cell r="E9" t="str">
-            <v/>
-          </cell>
-          <cell r="F9" t="str">
             <v/>
           </cell>
           <cell r="G9" t="str">
@@ -243,19 +225,10 @@
           <cell r="A10" t="str">
             <v/>
           </cell>
-          <cell r="B10" t="str">
-            <v>(0.0950)</v>
-          </cell>
           <cell r="C10" t="str">
             <v/>
           </cell>
           <cell r="D10" t="str">
-            <v/>
-          </cell>
-          <cell r="E10" t="str">
-            <v/>
-          </cell>
-          <cell r="F10" t="str">
             <v/>
           </cell>
           <cell r="G10" t="str">
@@ -266,19 +239,10 @@
           </cell>
         </row>
         <row r="12">
-          <cell r="B12" t="str">
-            <v>0.723***</v>
-          </cell>
           <cell r="C12" t="str">
             <v/>
           </cell>
           <cell r="D12" t="str">
-            <v/>
-          </cell>
-          <cell r="E12" t="str">
-            <v/>
-          </cell>
-          <cell r="F12" t="str">
             <v/>
           </cell>
           <cell r="G12" t="str">
@@ -292,21 +256,12 @@
           <cell r="A13" t="str">
             <v/>
           </cell>
-          <cell r="B13" t="str">
-            <v>(0.163)</v>
-          </cell>
           <cell r="C13" t="str">
             <v/>
           </cell>
           <cell r="D13" t="str">
             <v/>
           </cell>
-          <cell r="E13" t="str">
-            <v/>
-          </cell>
-          <cell r="F13" t="str">
-            <v/>
-          </cell>
           <cell r="G13" t="str">
             <v/>
           </cell>
@@ -315,19 +270,10 @@
           </cell>
         </row>
         <row r="15">
-          <cell r="B15" t="str">
-            <v>0.257</v>
-          </cell>
           <cell r="C15" t="str">
             <v/>
           </cell>
           <cell r="D15" t="str">
-            <v/>
-          </cell>
-          <cell r="E15" t="str">
-            <v/>
-          </cell>
-          <cell r="F15" t="str">
             <v/>
           </cell>
           <cell r="G15" t="str">
@@ -341,21 +287,12 @@
           <cell r="A16" t="str">
             <v/>
           </cell>
-          <cell r="B16" t="str">
-            <v>(0.189)</v>
-          </cell>
           <cell r="C16" t="str">
             <v/>
           </cell>
           <cell r="D16" t="str">
             <v/>
           </cell>
-          <cell r="E16" t="str">
-            <v/>
-          </cell>
-          <cell r="F16" t="str">
-            <v/>
-          </cell>
           <cell r="G16" t="str">
             <v/>
           </cell>
@@ -364,21 +301,12 @@
           </cell>
         </row>
         <row r="72">
-          <cell r="B72" t="str">
-            <v/>
-          </cell>
           <cell r="C72" t="str">
             <v>-0.0496</v>
           </cell>
           <cell r="D72" t="str">
             <v>-0.0397</v>
           </cell>
-          <cell r="E72" t="str">
-            <v>-0.218</v>
-          </cell>
-          <cell r="F72" t="str">
-            <v>-0.213</v>
-          </cell>
           <cell r="G72" t="str">
             <v>-0.0410</v>
           </cell>
@@ -390,21 +318,12 @@
           <cell r="A73" t="str">
             <v/>
           </cell>
-          <cell r="B73" t="str">
-            <v/>
-          </cell>
           <cell r="C73" t="str">
             <v>(0.0410)</v>
           </cell>
           <cell r="D73" t="str">
             <v>(0.0389)</v>
           </cell>
-          <cell r="E73" t="str">
-            <v>(0.168)</v>
-          </cell>
-          <cell r="F73" t="str">
-            <v>(0.227)</v>
-          </cell>
           <cell r="G73" t="str">
             <v>(0.0401)</v>
           </cell>
@@ -413,21 +332,12 @@
           </cell>
         </row>
         <row r="75">
-          <cell r="B75" t="str">
-            <v/>
-          </cell>
           <cell r="C75" t="str">
             <v>-0.0604*</v>
           </cell>
           <cell r="D75" t="str">
             <v>-0.0130</v>
           </cell>
-          <cell r="E75" t="str">
-            <v>-0.279**</v>
-          </cell>
-          <cell r="F75" t="str">
-            <v>-0.0755</v>
-          </cell>
           <cell r="G75" t="str">
             <v>-0.0878***</v>
           </cell>
@@ -439,21 +349,12 @@
           <cell r="A76" t="str">
             <v/>
           </cell>
-          <cell r="B76" t="str">
-            <v/>
-          </cell>
           <cell r="C76" t="str">
             <v>(0.0312)</v>
           </cell>
           <cell r="D76" t="str">
             <v>(0.0295)</v>
           </cell>
-          <cell r="E76" t="str">
-            <v>(0.135)</v>
-          </cell>
-          <cell r="F76" t="str">
-            <v>(0.167)</v>
-          </cell>
           <cell r="G76" t="str">
             <v>(0.0317)</v>
           </cell>
@@ -462,21 +363,12 @@
           </cell>
         </row>
         <row r="78">
-          <cell r="B78" t="str">
-            <v/>
-          </cell>
           <cell r="C78" t="str">
             <v>-0.0471</v>
           </cell>
           <cell r="D78" t="str">
             <v>-0.0423</v>
           </cell>
-          <cell r="E78" t="str">
-            <v>-0.226</v>
-          </cell>
-          <cell r="F78" t="str">
-            <v>-0.272</v>
-          </cell>
           <cell r="G78" t="str">
             <v>-0.0474</v>
           </cell>
@@ -488,21 +380,12 @@
           <cell r="A79" t="str">
             <v/>
           </cell>
-          <cell r="B79" t="str">
-            <v/>
-          </cell>
           <cell r="C79" t="str">
             <v>(0.0398)</v>
           </cell>
           <cell r="D79" t="str">
             <v>(0.0389)</v>
           </cell>
-          <cell r="E79" t="str">
-            <v>(0.159)</v>
-          </cell>
-          <cell r="F79" t="str">
-            <v>(0.220)</v>
-          </cell>
           <cell r="G79" t="str">
             <v>(0.0376)</v>
           </cell>
@@ -511,21 +394,12 @@
           </cell>
         </row>
         <row r="81">
-          <cell r="B81" t="str">
-            <v/>
-          </cell>
           <cell r="C81" t="str">
             <v>-0.0744**</v>
           </cell>
           <cell r="D81" t="str">
             <v>-0.0311</v>
           </cell>
-          <cell r="E81" t="str">
-            <v>-0.354**</v>
-          </cell>
-          <cell r="F81" t="str">
-            <v>-0.189</v>
-          </cell>
           <cell r="G81" t="str">
             <v>-0.0649*</v>
           </cell>
@@ -537,21 +411,12 @@
           <cell r="A82" t="str">
             <v/>
           </cell>
-          <cell r="B82" t="str">
-            <v/>
-          </cell>
           <cell r="C82" t="str">
             <v>(0.0321)</v>
           </cell>
           <cell r="D82" t="str">
             <v>(0.0298)</v>
           </cell>
-          <cell r="E82" t="str">
-            <v>(0.141)</v>
-          </cell>
-          <cell r="F82" t="str">
-            <v>(0.172)</v>
-          </cell>
           <cell r="G82" t="str">
             <v>(0.0334)</v>
           </cell>
@@ -560,21 +425,12 @@
           </cell>
         </row>
         <row r="84">
-          <cell r="B84" t="str">
-            <v/>
-          </cell>
           <cell r="C84" t="str">
             <v>-0.0904**</v>
           </cell>
           <cell r="D84" t="str">
             <v>-0.0440</v>
           </cell>
-          <cell r="E84" t="str">
-            <v>-0.412**</v>
-          </cell>
-          <cell r="F84" t="str">
-            <v>-0.264</v>
-          </cell>
           <cell r="G84" t="str">
             <v>-0.129***</v>
           </cell>
@@ -586,21 +442,12 @@
           <cell r="A85" t="str">
             <v/>
           </cell>
-          <cell r="B85" t="str">
-            <v/>
-          </cell>
           <cell r="C85" t="str">
             <v>(0.0414)</v>
           </cell>
           <cell r="D85" t="str">
             <v>(0.0417)</v>
           </cell>
-          <cell r="E85" t="str">
-            <v>(0.176)</v>
-          </cell>
-          <cell r="F85" t="str">
-            <v>(0.218)</v>
-          </cell>
           <cell r="G85" t="str">
             <v>(0.0406)</v>
           </cell>
@@ -609,21 +456,12 @@
           </cell>
         </row>
         <row r="87">
-          <cell r="B87" t="str">
-            <v/>
-          </cell>
           <cell r="C87" t="str">
             <v>-0.0648*</v>
           </cell>
           <cell r="D87" t="str">
             <v>-0.0248</v>
           </cell>
-          <cell r="E87" t="str">
-            <v>-0.301**</v>
-          </cell>
-          <cell r="F87" t="str">
-            <v>-0.182</v>
-          </cell>
           <cell r="G87" t="str">
             <v>-0.0419</v>
           </cell>
@@ -635,21 +473,12 @@
           <cell r="A88" t="str">
             <v/>
           </cell>
-          <cell r="B88" t="str">
-            <v/>
-          </cell>
           <cell r="C88" t="str">
             <v>(0.0373)</v>
           </cell>
           <cell r="D88" t="str">
             <v>(0.0380)</v>
           </cell>
-          <cell r="E88" t="str">
-            <v>(0.152)</v>
-          </cell>
-          <cell r="F88" t="str">
-            <v>(0.201)</v>
-          </cell>
           <cell r="G88" t="str">
             <v>(0.0353)</v>
           </cell>
@@ -658,21 +487,12 @@
           </cell>
         </row>
         <row r="90">
-          <cell r="B90" t="str">
-            <v/>
-          </cell>
           <cell r="C90" t="str">
             <v>0.306**</v>
           </cell>
           <cell r="D90" t="str">
             <v>0.293*</v>
           </cell>
-          <cell r="E90" t="str">
-            <v>0.672*</v>
-          </cell>
-          <cell r="F90" t="str">
-            <v>0.654</v>
-          </cell>
           <cell r="G90" t="str">
             <v>-0.0142</v>
           </cell>
@@ -684,21 +504,12 @@
           <cell r="A91" t="str">
             <v/>
           </cell>
-          <cell r="B91" t="str">
-            <v/>
-          </cell>
           <cell r="C91" t="str">
             <v>(0.137)</v>
           </cell>
           <cell r="D91" t="str">
             <v>(0.155)</v>
           </cell>
-          <cell r="E91" t="str">
-            <v>(0.395)</v>
-          </cell>
-          <cell r="F91" t="str">
-            <v>(0.427)</v>
-          </cell>
           <cell r="G91" t="str">
             <v>(0.122)</v>
           </cell>
@@ -707,20 +518,11 @@
           </cell>
         </row>
         <row r="96">
-          <cell r="B96" t="str">
-            <v>1700</v>
-          </cell>
           <cell r="C96" t="str">
             <v>1723</v>
           </cell>
           <cell r="D96" t="str">
             <v>1401</v>
-          </cell>
-          <cell r="E96" t="str">
-            <v>1700</v>
-          </cell>
-          <cell r="F96" t="str">
-            <v>1348</v>
           </cell>
           <cell r="G96" t="str">
             <v>1732</v>
@@ -744,42 +546,21 @@
           <cell r="A98" t="str">
             <v>Control Mean</v>
           </cell>
-          <cell r="B98" t="str">
-            <v>0.116</v>
-          </cell>
           <cell r="G98" t="str">
             <v>0.174</v>
           </cell>
         </row>
         <row r="99">
-          <cell r="B99" t="str">
-            <v>0.149</v>
-          </cell>
-          <cell r="E99" t="str">
-            <v>0.0870</v>
-          </cell>
-          <cell r="F99" t="str">
-            <v>0.119</v>
-          </cell>
           <cell r="H99" t="str">
             <v>0.0427</v>
           </cell>
         </row>
         <row r="100">
-          <cell r="B100" t="str">
-            <v/>
-          </cell>
           <cell r="C100" t="str">
             <v>0.0323</v>
           </cell>
           <cell r="D100" t="str">
             <v>0.191</v>
-          </cell>
-          <cell r="E100" t="str">
-            <v>0.0331</v>
-          </cell>
-          <cell r="F100" t="str">
-            <v>0.202</v>
           </cell>
           <cell r="G100" t="str">
             <v>0.0670</v>
@@ -1091,917 +872,585 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{853FBDF2-0918-4752-BC05-230A196258A9}">
-  <dimension ref="A3:K32"/>
+  <dimension ref="A3:F32"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.7265625" style="2"/>
-    <col min="3" max="3" width="2.453125" style="2" customWidth="1"/>
-    <col min="4" max="5" width="8.7265625" style="2"/>
-    <col min="6" max="6" width="3.08984375" style="2" customWidth="1"/>
-    <col min="7" max="8" width="8.7265625" style="2"/>
-    <col min="9" max="9" width="3.36328125" style="2" customWidth="1"/>
-    <col min="10" max="11" width="8.7265625" style="2"/>
+    <col min="2" max="3" width="8.7265625" style="2"/>
+    <col min="4" max="4" width="3.36328125" style="2" customWidth="1"/>
+    <col min="5" max="6" width="8.7265625" style="2"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" s="7"/>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="10"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
       <c r="F3" s="10"/>
-      <c r="G3" s="10"/>
-      <c r="H3" s="10"/>
-      <c r="I3" s="4"/>
-      <c r="J3" s="10" t="s">
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="B4" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="10"/>
+      <c r="E4" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="K3" s="10"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B4" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" s="3"/>
-      <c r="D4" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" s="10"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="H4" s="10"/>
-      <c r="J4" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="K4" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="5" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="5" t="str">
         <f>[1]fs_treatment_effects!A2</f>
         <v/>
       </c>
-      <c r="B5" s="6" t="str">
-        <f>[1]fs_treatment_effects!B2</f>
-        <v>(1)</v>
-      </c>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6" t="str">
-        <f>[1]fs_treatment_effects!C2</f>
-        <v>(2)</v>
-      </c>
-      <c r="E5" s="6" t="str">
-        <f>[1]fs_treatment_effects!D2</f>
-        <v>(3)</v>
-      </c>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6" t="str">
-        <f>[1]fs_treatment_effects!E2</f>
-        <v>(4)</v>
-      </c>
-      <c r="H5" s="6" t="str">
-        <f>[1]fs_treatment_effects!F2</f>
-        <v>(5)</v>
-      </c>
-      <c r="I5" s="6"/>
-      <c r="J5" s="6" t="str">
-        <f>[1]fs_treatment_effects!G2</f>
-        <v>(6)</v>
-      </c>
-      <c r="K5" s="6" t="str">
-        <f>[1]fs_treatment_effects!H2</f>
-        <v>(7)</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.35">
+      <c r="B5" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="6"/>
+      <c r="E5" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>4</v>
       </c>
       <c r="B6" s="2" t="str">
-        <f>[1]fs_treatment_effects!B9</f>
-        <v>0.121</v>
-      </c>
-      <c r="D6" s="2" t="str">
         <f>[1]fs_treatment_effects!C9</f>
         <v/>
       </c>
+      <c r="C6" s="2" t="str">
+        <f>[1]fs_treatment_effects!D9</f>
+        <v/>
+      </c>
       <c r="E6" s="2" t="str">
-        <f>[1]fs_treatment_effects!D9</f>
-        <v/>
-      </c>
-      <c r="G6" s="2" t="str">
-        <f>[1]fs_treatment_effects!E9</f>
-        <v/>
-      </c>
-      <c r="H6" s="2" t="str">
-        <f>[1]fs_treatment_effects!F9</f>
-        <v/>
-      </c>
-      <c r="J6" s="2" t="str">
         <f>[1]fs_treatment_effects!G9</f>
         <v>0.0288</v>
       </c>
-      <c r="K6" s="2" t="str">
+      <c r="F6" s="2" t="str">
         <f>[1]fs_treatment_effects!H9</f>
         <v>0.108</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="str">
         <f>[1]fs_treatment_effects!A10</f>
         <v/>
       </c>
       <c r="B7" s="2" t="str">
-        <f>[1]fs_treatment_effects!B10</f>
-        <v>(0.0950)</v>
-      </c>
-      <c r="D7" s="2" t="str">
         <f>[1]fs_treatment_effects!C10</f>
         <v/>
       </c>
+      <c r="C7" s="2" t="str">
+        <f>[1]fs_treatment_effects!D10</f>
+        <v/>
+      </c>
       <c r="E7" s="2" t="str">
-        <f>[1]fs_treatment_effects!D10</f>
-        <v/>
-      </c>
-      <c r="G7" s="2" t="str">
-        <f>[1]fs_treatment_effects!E10</f>
-        <v/>
-      </c>
-      <c r="H7" s="2" t="str">
-        <f>[1]fs_treatment_effects!F10</f>
-        <v/>
-      </c>
-      <c r="J7" s="2" t="str">
         <f>[1]fs_treatment_effects!G10</f>
         <v>(0.0175)</v>
       </c>
-      <c r="K7" s="2" t="str">
+      <c r="F7" s="2" t="str">
         <f>[1]fs_treatment_effects!H10</f>
         <v>(0.0680)</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>3</v>
       </c>
       <c r="B8" s="2" t="str">
-        <f>[1]fs_treatment_effects!B12</f>
-        <v>0.723***</v>
-      </c>
-      <c r="D8" s="2" t="str">
         <f>[1]fs_treatment_effects!C12</f>
         <v/>
       </c>
+      <c r="C8" s="2" t="str">
+        <f>[1]fs_treatment_effects!D12</f>
+        <v/>
+      </c>
       <c r="E8" s="2" t="str">
-        <f>[1]fs_treatment_effects!D12</f>
-        <v/>
-      </c>
-      <c r="G8" s="2" t="str">
-        <f>[1]fs_treatment_effects!E12</f>
-        <v/>
-      </c>
-      <c r="H8" s="2" t="str">
-        <f>[1]fs_treatment_effects!F12</f>
-        <v/>
-      </c>
-      <c r="J8" s="2" t="str">
         <f>[1]fs_treatment_effects!G12</f>
         <v/>
       </c>
-      <c r="K8" s="2" t="str">
+      <c r="F8" s="2" t="str">
         <f>[1]fs_treatment_effects!H12</f>
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="str">
         <f>[1]fs_treatment_effects!A13</f>
         <v/>
       </c>
       <c r="B9" s="2" t="str">
-        <f>[1]fs_treatment_effects!B13</f>
-        <v>(0.163)</v>
-      </c>
-      <c r="D9" s="2" t="str">
         <f>[1]fs_treatment_effects!C13</f>
         <v/>
       </c>
+      <c r="C9" s="2" t="str">
+        <f>[1]fs_treatment_effects!D13</f>
+        <v/>
+      </c>
       <c r="E9" s="2" t="str">
-        <f>[1]fs_treatment_effects!D13</f>
-        <v/>
-      </c>
-      <c r="G9" s="2" t="str">
-        <f>[1]fs_treatment_effects!E13</f>
-        <v/>
-      </c>
-      <c r="H9" s="2" t="str">
-        <f>[1]fs_treatment_effects!F13</f>
-        <v/>
-      </c>
-      <c r="J9" s="2" t="str">
         <f>[1]fs_treatment_effects!G13</f>
         <v/>
       </c>
-      <c r="K9" s="2" t="str">
+      <c r="F9" s="2" t="str">
         <f>[1]fs_treatment_effects!H13</f>
         <v/>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>2</v>
       </c>
       <c r="B10" s="2" t="str">
-        <f>[1]fs_treatment_effects!B15</f>
-        <v>0.257</v>
-      </c>
-      <c r="D10" s="2" t="str">
         <f>[1]fs_treatment_effects!C15</f>
         <v/>
       </c>
+      <c r="C10" s="2" t="str">
+        <f>[1]fs_treatment_effects!D15</f>
+        <v/>
+      </c>
       <c r="E10" s="2" t="str">
-        <f>[1]fs_treatment_effects!D15</f>
-        <v/>
-      </c>
-      <c r="G10" s="2" t="str">
-        <f>[1]fs_treatment_effects!E15</f>
-        <v/>
-      </c>
-      <c r="H10" s="2" t="str">
-        <f>[1]fs_treatment_effects!F15</f>
-        <v/>
-      </c>
-      <c r="J10" s="2" t="str">
         <f>[1]fs_treatment_effects!G15</f>
         <v/>
       </c>
-      <c r="K10" s="2" t="str">
+      <c r="F10" s="2" t="str">
         <f>[1]fs_treatment_effects!H15</f>
         <v/>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="str">
         <f>[1]fs_treatment_effects!A16</f>
         <v/>
       </c>
       <c r="B11" s="2" t="str">
-        <f>[1]fs_treatment_effects!B16</f>
-        <v>(0.189)</v>
-      </c>
-      <c r="D11" s="2" t="str">
         <f>[1]fs_treatment_effects!C16</f>
         <v/>
       </c>
+      <c r="C11" s="2" t="str">
+        <f>[1]fs_treatment_effects!D16</f>
+        <v/>
+      </c>
       <c r="E11" s="2" t="str">
-        <f>[1]fs_treatment_effects!D16</f>
-        <v/>
-      </c>
-      <c r="G11" s="2" t="str">
-        <f>[1]fs_treatment_effects!E16</f>
-        <v/>
-      </c>
-      <c r="H11" s="2" t="str">
-        <f>[1]fs_treatment_effects!F16</f>
-        <v/>
-      </c>
-      <c r="J11" s="2" t="str">
         <f>[1]fs_treatment_effects!G16</f>
         <v/>
       </c>
-      <c r="K11" s="2" t="str">
+      <c r="F11" s="2" t="str">
         <f>[1]fs_treatment_effects!H16</f>
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" s="1">
         <v>0.39583333333333331</v>
       </c>
       <c r="B12" s="2" t="str">
-        <f>[1]fs_treatment_effects!B72</f>
-        <v/>
-      </c>
-      <c r="D12" s="2" t="str">
         <f>[1]fs_treatment_effects!C72</f>
         <v>-0.0496</v>
       </c>
-      <c r="E12" s="2" t="str">
+      <c r="C12" s="2" t="str">
         <f>[1]fs_treatment_effects!D72</f>
         <v>-0.0397</v>
       </c>
-      <c r="G12" s="2" t="str">
-        <f>[1]fs_treatment_effects!E72</f>
-        <v>-0.218</v>
-      </c>
-      <c r="H12" s="2" t="str">
-        <f>[1]fs_treatment_effects!F72</f>
-        <v>-0.213</v>
-      </c>
-      <c r="J12" s="2" t="str">
+      <c r="E12" s="2" t="str">
         <f>[1]fs_treatment_effects!G72</f>
         <v>-0.0410</v>
       </c>
-      <c r="K12" s="2" t="str">
+      <c r="F12" s="2" t="str">
         <f>[1]fs_treatment_effects!H72</f>
         <v>-0.133</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="str">
         <f>[1]fs_treatment_effects!A73</f>
         <v/>
       </c>
       <c r="B13" s="2" t="str">
-        <f>[1]fs_treatment_effects!B73</f>
-        <v/>
-      </c>
-      <c r="D13" s="2" t="str">
         <f>[1]fs_treatment_effects!C73</f>
         <v>(0.0410)</v>
       </c>
-      <c r="E13" s="2" t="str">
+      <c r="C13" s="2" t="str">
         <f>[1]fs_treatment_effects!D73</f>
         <v>(0.0389)</v>
       </c>
-      <c r="G13" s="2" t="str">
-        <f>[1]fs_treatment_effects!E73</f>
-        <v>(0.168)</v>
-      </c>
-      <c r="H13" s="2" t="str">
-        <f>[1]fs_treatment_effects!F73</f>
-        <v>(0.227)</v>
-      </c>
-      <c r="J13" s="2" t="str">
+      <c r="E13" s="2" t="str">
         <f>[1]fs_treatment_effects!G73</f>
         <v>(0.0401)</v>
       </c>
-      <c r="K13" s="2" t="str">
+      <c r="F13" s="2" t="str">
         <f>[1]fs_treatment_effects!H73</f>
         <v>(0.138)</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" s="1">
         <v>0.41666666666666669</v>
       </c>
       <c r="B14" s="2" t="str">
-        <f>[1]fs_treatment_effects!B75</f>
-        <v/>
-      </c>
-      <c r="D14" s="2" t="str">
         <f>[1]fs_treatment_effects!C75</f>
         <v>-0.0604*</v>
       </c>
-      <c r="E14" s="2" t="str">
+      <c r="C14" s="2" t="str">
         <f>[1]fs_treatment_effects!D75</f>
         <v>-0.0130</v>
       </c>
-      <c r="G14" s="2" t="str">
-        <f>[1]fs_treatment_effects!E75</f>
-        <v>-0.279**</v>
-      </c>
-      <c r="H14" s="2" t="str">
-        <f>[1]fs_treatment_effects!F75</f>
-        <v>-0.0755</v>
-      </c>
-      <c r="J14" s="2" t="str">
+      <c r="E14" s="2" t="str">
         <f>[1]fs_treatment_effects!G75</f>
         <v>-0.0878***</v>
       </c>
-      <c r="K14" s="2" t="str">
+      <c r="F14" s="2" t="str">
         <f>[1]fs_treatment_effects!H75</f>
         <v>-0.326***</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="str">
         <f>[1]fs_treatment_effects!A76</f>
         <v/>
       </c>
       <c r="B15" s="2" t="str">
-        <f>[1]fs_treatment_effects!B76</f>
-        <v/>
-      </c>
-      <c r="D15" s="2" t="str">
         <f>[1]fs_treatment_effects!C76</f>
         <v>(0.0312)</v>
       </c>
-      <c r="E15" s="2" t="str">
+      <c r="C15" s="2" t="str">
         <f>[1]fs_treatment_effects!D76</f>
         <v>(0.0295)</v>
       </c>
-      <c r="G15" s="2" t="str">
-        <f>[1]fs_treatment_effects!E76</f>
-        <v>(0.135)</v>
-      </c>
-      <c r="H15" s="2" t="str">
-        <f>[1]fs_treatment_effects!F76</f>
-        <v>(0.167)</v>
-      </c>
-      <c r="J15" s="2" t="str">
+      <c r="E15" s="2" t="str">
         <f>[1]fs_treatment_effects!G76</f>
         <v>(0.0317)</v>
       </c>
-      <c r="K15" s="2" t="str">
+      <c r="F15" s="2" t="str">
         <f>[1]fs_treatment_effects!H76</f>
         <v>(0.115)</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" s="1">
         <v>0.4375</v>
       </c>
       <c r="B16" s="2" t="str">
-        <f>[1]fs_treatment_effects!B78</f>
-        <v/>
-      </c>
-      <c r="D16" s="2" t="str">
         <f>[1]fs_treatment_effects!C78</f>
         <v>-0.0471</v>
       </c>
-      <c r="E16" s="2" t="str">
+      <c r="C16" s="2" t="str">
         <f>[1]fs_treatment_effects!D78</f>
         <v>-0.0423</v>
       </c>
-      <c r="G16" s="2" t="str">
-        <f>[1]fs_treatment_effects!E78</f>
-        <v>-0.226</v>
-      </c>
-      <c r="H16" s="2" t="str">
-        <f>[1]fs_treatment_effects!F78</f>
-        <v>-0.272</v>
-      </c>
-      <c r="J16" s="2" t="str">
+      <c r="E16" s="2" t="str">
         <f>[1]fs_treatment_effects!G78</f>
         <v>-0.0474</v>
       </c>
-      <c r="K16" s="2" t="str">
+      <c r="F16" s="2" t="str">
         <f>[1]fs_treatment_effects!H78</f>
         <v>-0.157</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" t="str">
         <f>[1]fs_treatment_effects!A79</f>
         <v/>
       </c>
       <c r="B17" s="2" t="str">
-        <f>[1]fs_treatment_effects!B79</f>
-        <v/>
-      </c>
-      <c r="D17" s="2" t="str">
         <f>[1]fs_treatment_effects!C79</f>
         <v>(0.0398)</v>
       </c>
-      <c r="E17" s="2" t="str">
+      <c r="C17" s="2" t="str">
         <f>[1]fs_treatment_effects!D79</f>
         <v>(0.0389)</v>
       </c>
-      <c r="G17" s="2" t="str">
-        <f>[1]fs_treatment_effects!E79</f>
-        <v>(0.159)</v>
-      </c>
-      <c r="H17" s="2" t="str">
-        <f>[1]fs_treatment_effects!F79</f>
-        <v>(0.220)</v>
-      </c>
-      <c r="J17" s="2" t="str">
+      <c r="E17" s="2" t="str">
         <f>[1]fs_treatment_effects!G79</f>
         <v>(0.0376)</v>
       </c>
-      <c r="K17" s="2" t="str">
+      <c r="F17" s="2" t="str">
         <f>[1]fs_treatment_effects!H79</f>
         <v>(0.131)</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" s="1">
         <v>0.45833333333333331</v>
       </c>
       <c r="B18" s="2" t="str">
-        <f>[1]fs_treatment_effects!B81</f>
-        <v/>
-      </c>
-      <c r="D18" s="2" t="str">
         <f>[1]fs_treatment_effects!C81</f>
         <v>-0.0744**</v>
       </c>
-      <c r="E18" s="2" t="str">
+      <c r="C18" s="2" t="str">
         <f>[1]fs_treatment_effects!D81</f>
         <v>-0.0311</v>
       </c>
-      <c r="G18" s="2" t="str">
-        <f>[1]fs_treatment_effects!E81</f>
-        <v>-0.354**</v>
-      </c>
-      <c r="H18" s="2" t="str">
-        <f>[1]fs_treatment_effects!F81</f>
-        <v>-0.189</v>
-      </c>
-      <c r="J18" s="2" t="str">
+      <c r="E18" s="2" t="str">
         <f>[1]fs_treatment_effects!G81</f>
         <v>-0.0649*</v>
       </c>
-      <c r="K18" s="2" t="str">
+      <c r="F18" s="2" t="str">
         <f>[1]fs_treatment_effects!H81</f>
         <v>-0.224*</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" t="str">
         <f>[1]fs_treatment_effects!A82</f>
         <v/>
       </c>
       <c r="B19" s="2" t="str">
-        <f>[1]fs_treatment_effects!B82</f>
-        <v/>
-      </c>
-      <c r="D19" s="2" t="str">
         <f>[1]fs_treatment_effects!C82</f>
         <v>(0.0321)</v>
       </c>
-      <c r="E19" s="2" t="str">
+      <c r="C19" s="2" t="str">
         <f>[1]fs_treatment_effects!D82</f>
         <v>(0.0298)</v>
       </c>
-      <c r="G19" s="2" t="str">
-        <f>[1]fs_treatment_effects!E82</f>
-        <v>(0.141)</v>
-      </c>
-      <c r="H19" s="2" t="str">
-        <f>[1]fs_treatment_effects!F82</f>
-        <v>(0.172)</v>
-      </c>
-      <c r="J19" s="2" t="str">
+      <c r="E19" s="2" t="str">
         <f>[1]fs_treatment_effects!G82</f>
         <v>(0.0334)</v>
       </c>
-      <c r="K19" s="2" t="str">
+      <c r="F19" s="2" t="str">
         <f>[1]fs_treatment_effects!H82</f>
         <v>(0.121)</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" s="1">
         <v>0.47916666666666669</v>
       </c>
       <c r="B20" s="2" t="str">
-        <f>[1]fs_treatment_effects!B84</f>
-        <v/>
-      </c>
-      <c r="D20" s="2" t="str">
         <f>[1]fs_treatment_effects!C84</f>
         <v>-0.0904**</v>
       </c>
-      <c r="E20" s="2" t="str">
+      <c r="C20" s="2" t="str">
         <f>[1]fs_treatment_effects!D84</f>
         <v>-0.0440</v>
       </c>
-      <c r="G20" s="2" t="str">
-        <f>[1]fs_treatment_effects!E84</f>
-        <v>-0.412**</v>
-      </c>
-      <c r="H20" s="2" t="str">
-        <f>[1]fs_treatment_effects!F84</f>
-        <v>-0.264</v>
-      </c>
-      <c r="J20" s="2" t="str">
+      <c r="E20" s="2" t="str">
         <f>[1]fs_treatment_effects!G84</f>
         <v>-0.129***</v>
       </c>
-      <c r="K20" s="2" t="str">
+      <c r="F20" s="2" t="str">
         <f>[1]fs_treatment_effects!H84</f>
         <v>-0.503***</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" t="str">
         <f>[1]fs_treatment_effects!A85</f>
         <v/>
       </c>
       <c r="B21" s="2" t="str">
-        <f>[1]fs_treatment_effects!B85</f>
-        <v/>
-      </c>
-      <c r="D21" s="2" t="str">
         <f>[1]fs_treatment_effects!C85</f>
         <v>(0.0414)</v>
       </c>
-      <c r="E21" s="2" t="str">
+      <c r="C21" s="2" t="str">
         <f>[1]fs_treatment_effects!D85</f>
         <v>(0.0417)</v>
       </c>
-      <c r="G21" s="2" t="str">
-        <f>[1]fs_treatment_effects!E85</f>
-        <v>(0.176)</v>
-      </c>
-      <c r="H21" s="2" t="str">
-        <f>[1]fs_treatment_effects!F85</f>
-        <v>(0.218)</v>
-      </c>
-      <c r="J21" s="2" t="str">
+      <c r="E21" s="2" t="str">
         <f>[1]fs_treatment_effects!G85</f>
         <v>(0.0406)</v>
       </c>
-      <c r="K21" s="2" t="str">
+      <c r="F21" s="2" t="str">
         <f>[1]fs_treatment_effects!H85</f>
         <v>(0.174)</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" s="1">
         <v>0.5</v>
       </c>
       <c r="B22" s="2" t="str">
-        <f>[1]fs_treatment_effects!B87</f>
-        <v/>
-      </c>
-      <c r="D22" s="2" t="str">
         <f>[1]fs_treatment_effects!C87</f>
         <v>-0.0648*</v>
       </c>
-      <c r="E22" s="2" t="str">
+      <c r="C22" s="2" t="str">
         <f>[1]fs_treatment_effects!D87</f>
         <v>-0.0248</v>
       </c>
-      <c r="G22" s="2" t="str">
-        <f>[1]fs_treatment_effects!E87</f>
-        <v>-0.301**</v>
-      </c>
-      <c r="H22" s="2" t="str">
-        <f>[1]fs_treatment_effects!F87</f>
-        <v>-0.182</v>
-      </c>
-      <c r="J22" s="2" t="str">
+      <c r="E22" s="2" t="str">
         <f>[1]fs_treatment_effects!G87</f>
         <v>-0.0419</v>
       </c>
-      <c r="K22" s="2" t="str">
+      <c r="F22" s="2" t="str">
         <f>[1]fs_treatment_effects!H87</f>
         <v>-0.138</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" t="str">
         <f>[1]fs_treatment_effects!A88</f>
         <v/>
       </c>
       <c r="B23" s="2" t="str">
-        <f>[1]fs_treatment_effects!B88</f>
-        <v/>
-      </c>
-      <c r="D23" s="2" t="str">
         <f>[1]fs_treatment_effects!C88</f>
         <v>(0.0373)</v>
       </c>
-      <c r="E23" s="2" t="str">
+      <c r="C23" s="2" t="str">
         <f>[1]fs_treatment_effects!D88</f>
         <v>(0.0380)</v>
       </c>
-      <c r="G23" s="2" t="str">
-        <f>[1]fs_treatment_effects!E88</f>
-        <v>(0.152)</v>
-      </c>
-      <c r="H23" s="2" t="str">
-        <f>[1]fs_treatment_effects!F88</f>
-        <v>(0.201)</v>
-      </c>
-      <c r="J23" s="2" t="str">
+      <c r="E23" s="2" t="str">
         <f>[1]fs_treatment_effects!G88</f>
         <v>(0.0353)</v>
       </c>
-      <c r="K23" s="2" t="str">
+      <c r="F23" s="2" t="str">
         <f>[1]fs_treatment_effects!H88</f>
         <v>(0.119)</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" s="1">
         <v>0.52083333333333337</v>
       </c>
       <c r="B24" s="2" t="str">
-        <f>[1]fs_treatment_effects!B90</f>
-        <v/>
-      </c>
-      <c r="D24" s="2" t="str">
         <f>[1]fs_treatment_effects!C90</f>
         <v>0.306**</v>
       </c>
-      <c r="E24" s="2" t="str">
+      <c r="C24" s="2" t="str">
         <f>[1]fs_treatment_effects!D90</f>
         <v>0.293*</v>
       </c>
-      <c r="G24" s="2" t="str">
-        <f>[1]fs_treatment_effects!E90</f>
-        <v>0.672*</v>
-      </c>
-      <c r="H24" s="2" t="str">
-        <f>[1]fs_treatment_effects!F90</f>
-        <v>0.654</v>
-      </c>
-      <c r="J24" s="2" t="str">
+      <c r="E24" s="2" t="str">
         <f>[1]fs_treatment_effects!G90</f>
         <v>-0.0142</v>
       </c>
-      <c r="K24" s="2" t="str">
+      <c r="F24" s="2" t="str">
         <f>[1]fs_treatment_effects!H90</f>
         <v>-0.0297</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" t="str">
         <f>[1]fs_treatment_effects!A91</f>
         <v/>
       </c>
       <c r="B25" s="2" t="str">
-        <f>[1]fs_treatment_effects!B91</f>
-        <v/>
-      </c>
-      <c r="D25" s="2" t="str">
         <f>[1]fs_treatment_effects!C91</f>
         <v>(0.137)</v>
       </c>
-      <c r="E25" s="2" t="str">
+      <c r="C25" s="2" t="str">
         <f>[1]fs_treatment_effects!D91</f>
         <v>(0.155)</v>
       </c>
-      <c r="G25" s="2" t="str">
-        <f>[1]fs_treatment_effects!E91</f>
-        <v>(0.395)</v>
-      </c>
-      <c r="H25" s="2" t="str">
-        <f>[1]fs_treatment_effects!F91</f>
-        <v>(0.427)</v>
-      </c>
-      <c r="J25" s="2" t="str">
+      <c r="E25" s="2" t="str">
         <f>[1]fs_treatment_effects!G91</f>
         <v>(0.122)</v>
       </c>
-      <c r="K25" s="2" t="str">
+      <c r="F25" s="2" t="str">
         <f>[1]fs_treatment_effects!H91</f>
         <v>(0.435)</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" s="7" t="s">
         <v>1</v>
       </c>
       <c r="B27" s="4" t="str">
-        <f>[1]fs_treatment_effects!B96</f>
-        <v>1700</v>
-      </c>
-      <c r="C27" s="4"/>
-      <c r="D27" s="4" t="str">
         <f>[1]fs_treatment_effects!C96</f>
         <v>1723</v>
       </c>
-      <c r="E27" s="4" t="str">
+      <c r="C27" s="4" t="str">
         <f>[1]fs_treatment_effects!D96</f>
         <v>1401</v>
       </c>
-      <c r="F27" s="4"/>
-      <c r="G27" s="4" t="str">
-        <f>[1]fs_treatment_effects!E96</f>
-        <v>1700</v>
-      </c>
-      <c r="H27" s="4" t="str">
-        <f>[1]fs_treatment_effects!F96</f>
-        <v>1348</v>
-      </c>
-      <c r="I27" s="4"/>
-      <c r="J27" s="4" t="str">
+      <c r="D27" s="4"/>
+      <c r="E27" s="4" t="str">
         <f>[1]fs_treatment_effects!G96</f>
         <v>1732</v>
       </c>
-      <c r="K27" s="4" t="str">
+      <c r="F27" s="4" t="str">
         <f>[1]fs_treatment_effects!H96</f>
         <v>1732</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>0</v>
       </c>
-      <c r="B28" s="3" t="str">
-        <f>[1]fs_treatment_effects!B99</f>
-        <v>0.149</v>
-      </c>
-      <c r="D28" s="2" t="str">
+      <c r="B28" s="2" t="str">
         <f>[1]fs_treatment_effects!C97</f>
         <v>0.080</v>
       </c>
-      <c r="E28" s="2" t="str">
+      <c r="C28" s="2" t="str">
         <f>[1]fs_treatment_effects!D97</f>
         <v>0.101</v>
       </c>
-      <c r="G28" s="3" t="str">
-        <f>[1]fs_treatment_effects!E99</f>
-        <v>0.0870</v>
-      </c>
-      <c r="H28" s="3" t="str">
-        <f>[1]fs_treatment_effects!F99</f>
-        <v>0.119</v>
-      </c>
-      <c r="J28" s="3" t="str">
+      <c r="E28" s="3" t="str">
         <f>[1]fs_treatment_effects!G97</f>
         <v>0.037</v>
       </c>
-      <c r="K28" s="3" t="str">
+      <c r="F28" s="3" t="str">
         <f>[1]fs_treatment_effects!H99</f>
         <v>0.0427</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" s="8" t="str">
         <f>[1]fs_treatment_effects!A98</f>
         <v>Control Mean</v>
       </c>
-      <c r="B29" s="11" t="str">
-        <f>[1]fs_treatment_effects!B98</f>
-        <v>0.116</v>
-      </c>
+      <c r="B29" s="11"/>
       <c r="C29" s="11"/>
-      <c r="D29" s="11"/>
-      <c r="E29" s="11"/>
-      <c r="F29" s="11"/>
-      <c r="G29" s="11"/>
-      <c r="H29" s="11"/>
-      <c r="I29" s="3"/>
-      <c r="J29" s="11" t="str">
+      <c r="D29" s="3"/>
+      <c r="E29" s="11" t="str">
         <f>[1]fs_treatment_effects!G98</f>
         <v>0.174</v>
       </c>
-      <c r="K29" s="11"/>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="F29" s="11"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" s="8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B30" s="3" t="str">
-        <f>[1]fs_treatment_effects!B100</f>
-        <v/>
-      </c>
-      <c r="D30" s="3" t="str">
         <f>[1]fs_treatment_effects!C100</f>
         <v>0.0323</v>
       </c>
-      <c r="E30" s="3" t="str">
+      <c r="C30" s="3" t="str">
         <f>[1]fs_treatment_effects!D100</f>
         <v>0.191</v>
       </c>
-      <c r="G30" s="3" t="str">
-        <f>[1]fs_treatment_effects!E100</f>
-        <v>0.0331</v>
-      </c>
-      <c r="H30" s="3" t="str">
-        <f>[1]fs_treatment_effects!F100</f>
-        <v>0.202</v>
-      </c>
-      <c r="I30" s="3"/>
-      <c r="J30" s="3" t="str">
+      <c r="D30" s="3"/>
+      <c r="E30" s="3" t="str">
         <f>[1]fs_treatment_effects!G100</f>
         <v>0.0670</v>
       </c>
-      <c r="K30" s="3" t="str">
+      <c r="F30" s="3" t="str">
         <f>[1]fs_treatment_effects!H100</f>
         <v>0.0844</v>
       </c>
     </row>
-    <row r="31" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A31" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B31" s="6"/>
-      <c r="C31" s="6"/>
+      <c r="C31" s="6" t="s">
+        <v>8</v>
+      </c>
       <c r="D31" s="6"/>
-      <c r="E31" s="6" t="s">
-        <v>9</v>
-      </c>
+      <c r="E31" s="6"/>
       <c r="F31" s="6"/>
-      <c r="G31" s="6"/>
-      <c r="H31" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="I31" s="6"/>
-      <c r="J31" s="6"/>
-      <c r="K31" s="6"/>
-    </row>
-    <row r="32" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
+    </row>
+    <row r="32" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="J3:K3"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="B29:H29"/>
-    <mergeCell ref="J29:K29"/>
+  <mergeCells count="5">
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="E3:F3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="E29:F29"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>